<commit_message>
updates for the Universal SIEM Asset ID
</commit_message>
<xml_diff>
--- a/sample-data-and-templates/Hardware/degthatnetwork-hardwareassetlist.xlsx
+++ b/sample-data-and-templates/Hardware/degthatnetwork-hardwareassetlist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dalebingham/soteria/OpenRMFPro/RMF-Files/Hardware/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dalebingham/soteria/OpenRMFPro/openrmfpro-automation/sample-data-and-templates/Hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD3086D-8C44-5945-80EF-723BE91437C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7ADCF90-5036-1041-9444-8000819A9BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="21460" yWindow="11180" windowWidth="29400" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="55">
   <si>
     <t>Operating System</t>
   </si>
@@ -170,6 +170,21 @@
   </si>
   <si>
     <t>00:0C:25:88:C9:7D</t>
+  </si>
+  <si>
+    <t>SIEM Asset Id</t>
+  </si>
+  <si>
+    <t>0f823a91-23bc-42e1-92a8-f5421c9a1014</t>
+  </si>
+  <si>
+    <t>0f823a91-23bc-42e1-92a8-f5421c9a1015</t>
+  </si>
+  <si>
+    <t>0f823a91-23bc-42e1-92a8-f5421c9a1017</t>
+  </si>
+  <si>
+    <t>0f823a91-23bc-42e1-92a8-f5421c9a1020</t>
   </si>
 </sst>
 </file>
@@ -228,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -242,6 +257,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -558,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" style="2" customWidth="1"/>
@@ -570,10 +588,11 @@
     <col min="11" max="11" width="38.140625" style="2" customWidth="1"/>
     <col min="12" max="12" width="26.5703125" style="2" customWidth="1"/>
     <col min="13" max="13" width="26.42578125" style="2" customWidth="1"/>
-    <col min="14" max="16384" width="10.7109375" style="2"/>
+    <col min="14" max="14" width="46.85546875" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="10.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -613,8 +632,11 @@
       <c r="M1" s="1" t="s">
         <v>34</v>
       </c>
+      <c r="N1" s="5" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -652,8 +674,11 @@
       <c r="M2" s="3" t="s">
         <v>36</v>
       </c>
+      <c r="N2" s="3" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -691,8 +716,9 @@
       <c r="M3" s="3" t="s">
         <v>44</v>
       </c>
+      <c r="N3" s="3"/>
     </row>
-    <row r="4" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
@@ -730,8 +756,11 @@
       <c r="M4" s="3" t="s">
         <v>45</v>
       </c>
+      <c r="N4" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="5" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -769,8 +798,9 @@
       <c r="M5" s="3" t="s">
         <v>36</v>
       </c>
+      <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -804,8 +834,9 @@
       </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
     </row>
-    <row r="7" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
@@ -843,8 +874,11 @@
       <c r="M7" s="3" t="s">
         <v>47</v>
       </c>
+      <c r="N7" s="3" t="s">
+        <v>53</v>
+      </c>
     </row>
-    <row r="8" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
@@ -880,8 +914,9 @@
       <c r="M8" s="3" t="s">
         <v>48</v>
       </c>
+      <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>18</v>
       </c>
@@ -917,8 +952,11 @@
       <c r="M9" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="N9" s="3" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="10" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>19</v>
       </c>
@@ -954,6 +992,7 @@
       <c r="M10" s="3" t="s">
         <v>46</v>
       </c>
+      <c r="N10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update for additional date fields for HW
</commit_message>
<xml_diff>
--- a/sample-data-and-templates/Hardware/degthatnetwork-hardwareassetlist.xlsx
+++ b/sample-data-and-templates/Hardware/degthatnetwork-hardwareassetlist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dalebingham/soteria/OpenRMFPro/openrmfpro-automation/sample-data-and-templates/Hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7ADCF90-5036-1041-9444-8000819A9BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D70ED03-70EF-774D-9275-B22E25BF799F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21460" yWindow="11180" windowWidth="29400" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21300" yWindow="11160" windowWidth="39180" windowHeight="17220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HardwareListing" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="57">
   <si>
     <t>Operating System</t>
   </si>
@@ -185,6 +185,12 @@
   </si>
   <si>
     <t>0f823a91-23bc-42e1-92a8-f5421c9a1020</t>
+  </si>
+  <si>
+    <t>Purchase Date</t>
+  </si>
+  <si>
+    <t>Install Date</t>
   </si>
 </sst>
 </file>
@@ -243,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -259,8 +265,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -576,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" style="2" customWidth="1"/>
@@ -589,10 +598,11 @@
     <col min="12" max="12" width="26.5703125" style="2" customWidth="1"/>
     <col min="13" max="13" width="26.42578125" style="2" customWidth="1"/>
     <col min="14" max="14" width="46.85546875" style="2" customWidth="1"/>
-    <col min="15" max="16384" width="10.7109375" style="2"/>
+    <col min="15" max="16" width="19.7109375" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="10.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -632,11 +642,17 @@
       <c r="M1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="O1" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>56</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" ht="20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="20" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -674,11 +690,11 @@
       <c r="M2" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="N2" s="3" t="s">
-        <v>51</v>
-      </c>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
     </row>
-    <row r="3" spans="1:14" ht="20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="20" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -716,9 +732,17 @@
       <c r="M3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="N3" s="3"/>
+      <c r="N3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="O3" s="6">
+        <v>45323</v>
+      </c>
+      <c r="P3" s="6">
+        <v>45366</v>
+      </c>
     </row>
-    <row r="4" spans="1:14" ht="20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="20" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
@@ -756,11 +780,11 @@
       <c r="M4" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="N4" s="3" t="s">
-        <v>52</v>
-      </c>
+      <c r="N4" s="3"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
     </row>
-    <row r="5" spans="1:14" ht="20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="20" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -798,9 +822,13 @@
       <c r="M5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="N5" s="3"/>
+      <c r="N5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
     </row>
-    <row r="6" spans="1:14" ht="20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="20" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -835,8 +863,10 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
     </row>
-    <row r="7" spans="1:14" ht="20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="20" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
@@ -874,11 +904,11 @@
       <c r="M7" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="N7" s="3" t="s">
-        <v>53</v>
-      </c>
+      <c r="N7" s="3"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
     </row>
-    <row r="8" spans="1:14" ht="20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="20" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
@@ -914,9 +944,13 @@
       <c r="M8" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="N8" s="3"/>
+      <c r="N8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
     </row>
-    <row r="9" spans="1:14" ht="20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="20" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>18</v>
       </c>
@@ -952,11 +986,11 @@
       <c r="M9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="N9" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="N9" s="3"/>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
     </row>
-    <row r="10" spans="1:14" ht="20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="20" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>19</v>
       </c>
@@ -992,7 +1026,11 @@
       <c r="M10" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="N10" s="3"/>
+      <c r="N10" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>